<commit_message>
Refactor transient coefficient tests for clarity and accuracy
</commit_message>
<xml_diff>
--- a/productiecapaciteit/results/Wvptweerstand/Wvptweerstand_modelcoefficienten.xlsx
+++ b/productiecapaciteit/results/Wvptweerstand/Wvptweerstand_modelcoefficienten.xlsx
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38020965748</v>
+        <v>46200.38020965278</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38285495128</v>
+        <v>46200.38285495371</v>
       </c>
     </row>
   </sheetData>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38315274779</v>
+        <v>46200.38315274305</v>
       </c>
     </row>
   </sheetData>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38365194615</v>
+        <v>46200.38365194444</v>
       </c>
     </row>
   </sheetData>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38377106741</v>
+        <v>46200.38377106481</v>
       </c>
     </row>
   </sheetData>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38386960846</v>
+        <v>46200.38386960648</v>
       </c>
     </row>
   </sheetData>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38397108745</v>
+        <v>46200.38397108796</v>
       </c>
     </row>
   </sheetData>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38408188878</v>
+        <v>46200.38408188657</v>
       </c>
     </row>
   </sheetData>
@@ -1707,7 +1707,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38421917913</v>
+        <v>46200.38421917824</v>
       </c>
     </row>
   </sheetData>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>43.59614672007761</v>
+        <v>43.59566385278046</v>
       </c>
     </row>
     <row r="3">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>219.352658763325</v>
+        <v>219.3429509924534</v>
       </c>
     </row>
     <row r="13">
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38426850313</v>
+        <v>46202.43523520969</v>
       </c>
     </row>
   </sheetData>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38442649734</v>
+        <v>46200.38442649305</v>
       </c>
     </row>
   </sheetData>
@@ -2130,7 +2130,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38067107986</v>
+        <v>46200.38067107639</v>
       </c>
     </row>
   </sheetData>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38451594578</v>
+        <v>46200.38451594907</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38463738448</v>
+        <v>46200.38463738426</v>
       </c>
     </row>
   </sheetData>
@@ -2553,7 +2553,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38471892442</v>
+        <v>46200.38471892361</v>
       </c>
     </row>
   </sheetData>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38481662687</v>
+        <v>46200.38481663194</v>
       </c>
     </row>
   </sheetData>
@@ -2835,7 +2835,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38487244416</v>
+        <v>46200.38487244213</v>
       </c>
     </row>
   </sheetData>
@@ -2976,7 +2976,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38095323743</v>
+        <v>46200.38095324074</v>
       </c>
     </row>
   </sheetData>
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38138425728</v>
+        <v>46200.38138425926</v>
       </c>
     </row>
   </sheetData>
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38159058958</v>
+        <v>46200.38159059028</v>
       </c>
     </row>
   </sheetData>
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38189980573</v>
+        <v>46200.38189980324</v>
       </c>
     </row>
   </sheetData>
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38222395335</v>
+        <v>46200.38222395833</v>
       </c>
     </row>
   </sheetData>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38242336587</v>
+        <v>46200.38242336806</v>
       </c>
     </row>
   </sheetData>
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46200.38261160292</v>
+        <v>46200.38261159722</v>
       </c>
     </row>
   </sheetData>

</xml_diff>